<commit_message>
Added Cost Estimation metrics (Scrum Calculations)
</commit_message>
<xml_diff>
--- a/Documentation and Diagrams/Cost_Estimation_Metrics.xlsx
+++ b/Documentation and Diagrams/Cost_Estimation_Metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://livecoventryac-my.sharepoint.com/personal/mohame219_uni_coventry_ac_uk/Documents/SOFTWARE ENGINEERING PROJECT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1879139A-066F-8E41-B388-64670522C860}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{1879139A-066F-8E41-B388-64670522C860}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6AC6010F-CE58-BA40-B64F-018D41956665}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{56A60C74-3EA1-E045-B2DA-0517CDF3D209}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="127">
   <si>
     <t>Function Point Calculation</t>
   </si>
@@ -452,9 +452,6 @@
   </si>
   <si>
     <t>The system achieved a Defect Removal Efficiency (DRE) of 90% demonstrating the effectiveness of testing conducted</t>
-  </si>
-  <si>
-    <t>Scores</t>
   </si>
   <si>
     <t>HTML = 48.9%</t>
@@ -2143,9 +2140,6 @@
         <v>9</v>
       </c>
       <c r="K7" s="6"/>
-      <c r="N7" t="s">
-        <v>118</v>
-      </c>
     </row>
     <row r="8" spans="2:34" ht="17" thickBot="1">
       <c r="B8" s="14"/>
@@ -3707,14 +3701,14 @@
       </c>
       <c r="D68" s="57"/>
       <c r="E68" s="86" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="F68" s="6"/>
     </row>
     <row r="69" spans="2:6">
       <c r="B69" s="14"/>
       <c r="C69" s="45" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D69" s="57"/>
       <c r="E69" s="87"/>
@@ -3723,7 +3717,7 @@
     <row r="70" spans="2:6">
       <c r="B70" s="14"/>
       <c r="C70" s="45" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D70" s="57"/>
       <c r="E70" s="87"/>
@@ -3732,7 +3726,7 @@
     <row r="71" spans="2:6">
       <c r="B71" s="14"/>
       <c r="C71" s="45" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D71" s="57"/>
       <c r="E71" s="87"/>
@@ -3741,7 +3735,7 @@
     <row r="72" spans="2:6" ht="17" thickBot="1">
       <c r="B72" s="14"/>
       <c r="C72" s="46" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D72" s="57"/>
       <c r="E72" s="87"/>
@@ -3905,7 +3899,7 @@
     <row r="89" spans="2:6">
       <c r="B89" s="16"/>
       <c r="C89" s="70" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D89" s="71"/>
       <c r="E89" s="72"/>
@@ -3957,7 +3951,7 @@
         <v>8</v>
       </c>
       <c r="E95" s="147" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="F95" s="6"/>
     </row>
@@ -4083,7 +4077,7 @@
       </c>
       <c r="D108" s="15"/>
       <c r="E108" s="147" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="109" spans="2:6">
@@ -4103,7 +4097,7 @@
     <row r="111" spans="2:6">
       <c r="B111" s="14"/>
       <c r="C111" s="15" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D111" s="15"/>
       <c r="E111" s="148"/>

</xml_diff>